<commit_message>
Modified component list for motor controller
</commit_message>
<xml_diff>
--- a/Regen-brake/Farnell_component_lists/Farnell_seznam_komponent.xlsx
+++ b/Regen-brake/Farnell_component_lists/Farnell_seznam_komponent.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\timli\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\timli\Documents\Solar-bot\Regen-brake\Farnell_component_lists\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2DAD72AF-1B85-4561-924C-9C8748B00423}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00EB4904-81DA-4B28-9304-8E0EF98EEB2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13728" yWindow="0" windowWidth="9408" windowHeight="13776" xr2:uid="{E5A601E2-56F0-4850-8D4B-4119E24A9517}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{E5A601E2-56F0-4850-8D4B-4119E24A9517}"/>
   </bookViews>
   <sheets>
     <sheet name="List1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="31">
   <si>
     <t>Količina</t>
   </si>
@@ -75,13 +75,70 @@
   </si>
   <si>
     <t>https://si.farnell.com/multicomp-pro/irf540n/mosfet-n-channel-100v-33a-to-220/dp/4472945</t>
+  </si>
+  <si>
+    <t>Opis</t>
+  </si>
+  <si>
+    <t>Brake resistor</t>
+  </si>
+  <si>
+    <t>jumpers</t>
+  </si>
+  <si>
+    <t>MCU</t>
+  </si>
+  <si>
+    <t>comparator</t>
+  </si>
+  <si>
+    <t>HI and LO side driver</t>
+  </si>
+  <si>
+    <t>diodes</t>
+  </si>
+  <si>
+    <t>fast diodes</t>
+  </si>
+  <si>
+    <t>LO side driver for brake</t>
+  </si>
+  <si>
+    <t>Mosfets</t>
+  </si>
+  <si>
+    <t>COMPONENTS FOR SOLAR BOT (NOT FINAL !)</t>
+  </si>
+  <si>
+    <t>COMPONENTS FOR DC MOTOR DRIVER</t>
+  </si>
+  <si>
+    <t>https://si.farnell.com/texas-instruments/cd74hc14e/ic-74hc-74hc14-dip14-6v/dp/3120195</t>
+  </si>
+  <si>
+    <t>Schmitt trigger</t>
+  </si>
+  <si>
+    <t>https://si.farnell.com/texas-instruments/sn74hc02n/ic-quad-2-input-nor-74hc02-dip14/dp/3120423</t>
+  </si>
+  <si>
+    <t>Quad NOR</t>
+  </si>
+  <si>
+    <t>https://si.farnell.com/infineon/ir2110spbf/ic-mosfet-driver-high-low-side/dp/8638845</t>
+  </si>
+  <si>
+    <t>https://si.farnell.com/stmicroelectronics/stm32f103c8t6/mcu-32bit-cortex-m3-72mhz-lqfp/dp/1447637</t>
+  </si>
+  <si>
+    <t>STM32F103C8T6</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -104,6 +161,43 @@
       <family val="2"/>
       <charset val="238"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF161616"/>
+      <name val="Aptos Display"/>
+      <family val="2"/>
+      <scheme val="major"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -113,7 +207,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="17">
     <border>
       <left/>
       <right/>
@@ -269,7 +363,7 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right style="thin">
+      <right style="medium">
         <color indexed="64"/>
       </right>
       <top style="medium">
@@ -284,9 +378,7 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
+      <right/>
       <top style="medium">
         <color indexed="64"/>
       </top>
@@ -295,11 +387,62 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -316,29 +459,69 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hiperpovezava" xfId="1" builtinId="8"/>
     <cellStyle name="Navadno" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -671,125 +854,268 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F87A3A8-AC20-4FA2-A372-6CECD75118CC}">
-  <dimension ref="B3:D13"/>
+  <dimension ref="B2:E23"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="16.88671875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="86" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="4" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="10" t="s">
+    <row r="2" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="D2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="4" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B4" s="9" t="s">
         <v>4</v>
       </c>
       <c r="C4" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="12" t="s">
+      <c r="D4" s="15" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B5" s="7">
+      <c r="E4" s="16" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B5" s="6">
         <v>9567305</v>
       </c>
-      <c r="C5" s="8">
+      <c r="C5" s="7">
         <v>2</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="D5" s="12" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="6" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="E5" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B6" s="2">
         <v>2834673</v>
       </c>
       <c r="C6" s="1">
         <v>50</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="13" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="7" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="E6" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B7" s="2">
         <v>2466939</v>
       </c>
       <c r="C7" s="1">
         <v>2</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="13" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="8" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="E7" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B8" s="2">
         <v>2824967</v>
       </c>
       <c r="C8" s="1">
         <v>5</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="9" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="E8" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B9" s="2">
-        <v>8638837</v>
+        <v>8638845</v>
       </c>
       <c r="C9" s="1">
-        <v>6</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="10" spans="2:4" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B10" s="2">
         <v>1776392</v>
       </c>
       <c r="C10" s="1">
         <v>20</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="11" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="E10" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B11" s="2">
         <v>1467502</v>
       </c>
       <c r="C11" s="1">
         <v>5</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="D11" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="12" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="E11" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="12" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B12" s="2">
         <v>1439711</v>
       </c>
       <c r="C12" s="1">
         <v>5</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="1" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="13" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E12" s="3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B13" s="4">
         <v>4472945</v>
       </c>
       <c r="C13" s="5">
         <v>15</v>
       </c>
-      <c r="D13" s="6" t="s">
+      <c r="D13" s="14" t="s">
         <v>11</v>
       </c>
+      <c r="E13" s="17" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="16" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D16" s="10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B17" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="C17" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="D17" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="E17" s="16" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="18" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B18" s="21">
+        <v>4472945</v>
+      </c>
+      <c r="C18" s="22">
+        <v>15</v>
+      </c>
+      <c r="D18" s="23" t="s">
+        <v>11</v>
+      </c>
+      <c r="E18" s="22" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="19" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B19" s="19">
+        <v>2834673</v>
+      </c>
+      <c r="C19" s="18">
+        <v>50</v>
+      </c>
+      <c r="D19" s="18" t="s">
+        <v>3</v>
+      </c>
+      <c r="E19" s="18" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="20" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B20" s="20">
+        <v>8638837</v>
+      </c>
+      <c r="C20" s="1">
+        <v>2</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="21" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B21" s="20">
+        <v>3120195</v>
+      </c>
+      <c r="C21" s="1">
+        <v>1</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="22" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B22" s="20">
+        <v>3120423</v>
+      </c>
+      <c r="C22" s="1">
+        <v>1</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="23" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B23" s="20">
+        <v>1447637</v>
+      </c>
+      <c r="C23" s="24">
+        <v>2</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E23" s="25" t="s">
+        <v>30</v>
+      </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D13" r:id="rId1" xr:uid="{9C8E1771-A730-44B3-97B3-54EE52F53D64}"/>
+    <hyperlink ref="D18" r:id="rId2" xr:uid="{2F79D4D2-C8ED-4FF7-AF6C-FF904E291606}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>